<commit_message>
fix: localize new buqi stage prefabs
</commit_message>
<xml_diff>
--- a/Design/Excel/Localization.xlsx
+++ b/Design/Excel/Localization.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1af74662fb4a4f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R096d4034927b490f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3377,35 +3377,147 @@
     </x:row>
     <x:row r="141">
       <x:c r="A141"/>
-      <x:c r="B141"/>
-      <x:c r="C141"/>
-      <x:c r="D141"/>
-      <x:c r="E141"/>
-      <x:c r="F141"/>
+      <x:c r="B141" t="str">
+        <x:v>Buqi.Stage.OperationChoice.Description</x:v>
+      </x:c>
+      <x:c r="C141" t="str">
+        <x:v>选择坊市、机缘或静修；当前周天保持可见。</x:v>
+      </x:c>
+      <x:c r="D141" t="str">
+        <x:v>Choose the bazaar, an encounter, or cultivation; the current cycle remains visible.</x:v>
+      </x:c>
+      <x:c r="E141" t="str">
+        <x:v>選擇坊市、機緣或靜修；目前周天保持可見。</x:v>
+      </x:c>
+      <x:c r="F141" t="str">
+        <x:v>상점, 기연 또는 수련을 선택하세요. 현재 주천은 계속 표시됩니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142"/>
-      <x:c r="B142"/>
-      <x:c r="C142"/>
-      <x:c r="D142"/>
-      <x:c r="E142"/>
-      <x:c r="F142"/>
+      <x:c r="B142" t="str">
+        <x:v>Buqi.Stage.OperationChoice.Title</x:v>
+      </x:c>
+      <x:c r="C142" t="str">
+        <x:v>经营选择</x:v>
+      </x:c>
+      <x:c r="D142" t="str">
+        <x:v>Operation Choice</x:v>
+      </x:c>
+      <x:c r="E142" t="str">
+        <x:v>經營選擇</x:v>
+      </x:c>
+      <x:c r="F142" t="str">
+        <x:v>운영 선택</x:v>
+      </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143"/>
-      <x:c r="B143"/>
-      <x:c r="C143"/>
-      <x:c r="D143"/>
-      <x:c r="E143"/>
-      <x:c r="F143"/>
+      <x:c r="B143" t="str">
+        <x:v>Buqi.Stage.PveSelection.Description</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>选择初阶、进阶或险阶后直接进入战斗。</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>Choose Novice, Advanced, or Perilous, then enter battle.</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>選擇初階、進階或險階後直接進入戰鬥。</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>초급, 중급 또는 위험 단계를 선택한 뒤 바로 전투에 진입하세요.</x:v>
+      </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144"/>
-      <x:c r="B144"/>
-      <x:c r="C144"/>
-      <x:c r="D144"/>
-      <x:c r="E144"/>
-      <x:c r="F144"/>
+      <x:c r="B144" t="str">
+        <x:v>Buqi.Stage.PveSelection.Title</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>PVE 选关</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>PVE Selection</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>PVE 選關</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>PVE 선택</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145"/>
+      <x:c r="B145" t="str">
+        <x:v>Buqi.Stage.TribulationRoute.Description</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>九日夜战后选择一条渡劫路线。</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>After the ninth night's battle, choose a tribulation route.</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>九日夜戰後選擇一條渡劫路線。</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>9일째 야간 전투 후 천겁 경로를 하나 선택하세요.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146"/>
+      <x:c r="B146" t="str">
+        <x:v>Buqi.Stage.TribulationRoute.Title</x:v>
+      </x:c>
+      <x:c r="C146" t="str">
+        <x:v>渡劫路线</x:v>
+      </x:c>
+      <x:c r="D146" t="str">
+        <x:v>Tribulation Route</x:v>
+      </x:c>
+      <x:c r="E146" t="str">
+        <x:v>渡劫路線</x:v>
+      </x:c>
+      <x:c r="F146" t="str">
+        <x:v>천겁 경로</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147"/>
+      <x:c r="B147" t="str">
+        <x:v>Buqi.Stage.TribulationStage.Description</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>应劫并推进当前阶段。</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>Face the tribulation and advance the current stage.</x:v>
+      </x:c>
+      <x:c r="E147" t="str">
+        <x:v>應劫並推進目前階段。</x:v>
+      </x:c>
+      <x:c r="F147" t="str">
+        <x:v>천겁에 맞서 현재 단계를 진행하세요.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148"/>
+      <x:c r="B148" t="str">
+        <x:v>Buqi.Stage.TribulationStage.Title</x:v>
+      </x:c>
+      <x:c r="C148" t="str">
+        <x:v>三阶段天劫</x:v>
+      </x:c>
+      <x:c r="D148" t="str">
+        <x:v>Three-Stage Tribulation</x:v>
+      </x:c>
+      <x:c r="E148" t="str">
+        <x:v>三階段天劫</x:v>
+      </x:c>
+      <x:c r="F148" t="str">
+        <x:v>3단계 천겁</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(buqi): finalize four-period demo flow UI
</commit_message>
<xml_diff>
--- a/Design/Excel/Localization.xlsx
+++ b/Design/Excel/Localization.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R096d4034927b490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rf1d4f81e9d79483e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3519,6 +3519,114 @@
         <x:v>3단계 천겁</x:v>
       </x:c>
     </x:row>
+    <x:row r="149">
+      <x:c r="A149"/>
+      <x:c r="B149" t="str">
+        <x:v>Buqi.RunShell.DayRecord</x:v>
+      </x:c>
+      <x:c r="C149" t="str">
+        <x:v>日记录</x:v>
+      </x:c>
+      <x:c r="D149" t="str">
+        <x:v>Day Record</x:v>
+      </x:c>
+      <x:c r="E149" t="str">
+        <x:v>日記錄</x:v>
+      </x:c>
+      <x:c r="F149" t="str">
+        <x:v>일일 기록</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150"/>
+      <x:c r="B150" t="str">
+        <x:v>Buqi.RunShell.MorningOperation</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>晨 · 经营</x:v>
+      </x:c>
+      <x:c r="D150" t="str">
+        <x:v>Morning · Operation</x:v>
+      </x:c>
+      <x:c r="E150" t="str">
+        <x:v>晨 · 經營</x:v>
+      </x:c>
+      <x:c r="F150" t="str">
+        <x:v>아침 · 경영</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151"/>
+      <x:c r="B151" t="str">
+        <x:v>Buqi.RunShell.NoonOperation</x:v>
+      </x:c>
+      <x:c r="C151" t="str">
+        <x:v>昼 · 经营</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>Noon · Operation</x:v>
+      </x:c>
+      <x:c r="E151" t="str">
+        <x:v>晝 · 經營</x:v>
+      </x:c>
+      <x:c r="F151" t="str">
+        <x:v>낮 · 경영</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152"/>
+      <x:c r="B152" t="str">
+        <x:v>Buqi.RunShell.DuskPve</x:v>
+      </x:c>
+      <x:c r="C152" t="str">
+        <x:v>昏 · PVE</x:v>
+      </x:c>
+      <x:c r="D152" t="str">
+        <x:v>Dusk · PVE</x:v>
+      </x:c>
+      <x:c r="E152" t="str">
+        <x:v>昏 · PVE</x:v>
+      </x:c>
+      <x:c r="F152" t="str">
+        <x:v>해질녘 · PVE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153"/>
+      <x:c r="B153" t="str">
+        <x:v>Buqi.RunShell.NightPvp</x:v>
+      </x:c>
+      <x:c r="C153" t="str">
+        <x:v>夜 · 异步 PVP</x:v>
+      </x:c>
+      <x:c r="D153" t="str">
+        <x:v>Night · Async PVP</x:v>
+      </x:c>
+      <x:c r="E153" t="str">
+        <x:v>夜 · 非同步 PVP</x:v>
+      </x:c>
+      <x:c r="F153" t="str">
+        <x:v>밤 · 비동기 PVP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154"/>
+      <x:c r="B154" t="str">
+        <x:v>Buqi.Stage.Shared.CurrentBoard</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>当前周天</x:v>
+      </x:c>
+      <x:c r="D154" t="str">
+        <x:v>Current Cycle Board</x:v>
+      </x:c>
+      <x:c r="E154" t="str">
+        <x:v>當前周天</x:v>
+      </x:c>
+      <x:c r="F154" t="str">
+        <x:v>현재 주천</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>